<commit_message>
auto-push Tue 09/01/2026 16:42:32.22
</commit_message>
<xml_diff>
--- a/trader-scoreboard.bak-2026-09-01.xlsx
+++ b/trader-scoreboard.bak-2026-09-01.xlsx
@@ -17,7 +17,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="7">
+  <numFmts count="8">
     <numFmt numFmtId="164" formatCode="$#,##0;($#,##0);-"/>
     <numFmt numFmtId="165" formatCode="+0.0%;-0.0%"/>
     <numFmt numFmtId="166" formatCode="$#,##0.00;[Red]-$#,##0.00"/>
@@ -25,6 +25,7 @@
     <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0;[Red]-&quot;$&quot;#,##0"/>
     <numFmt numFmtId="169" formatCode="0.0%;[Red]-0.0%"/>
     <numFmt numFmtId="170" formatCode="$#,##0;[Red]-$#,##0"/>
+    <numFmt numFmtId="171" formatCode="#,##0.00;[Red]-#,##0.00"/>
   </numFmts>
   <fonts count="30">
     <font>
@@ -266,7 +267,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="57">
+  <cellXfs count="62">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -334,6 +335,13 @@
     <xf numFmtId="166" fontId="26" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="27" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="28" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="171" fontId="25" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="171" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="171" fontId="26" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -699,14 +707,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M40"/>
+  <dimension ref="A1:M44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="9" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
     <col width="11" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
@@ -718,67 +726,67 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="52" t="inlineStr">
+      <c r="A1" s="57" t="inlineStr">
         <is>
           <t>Caller</t>
         </is>
       </c>
-      <c r="B1" s="52" t="inlineStr">
+      <c r="B1" s="57" t="inlineStr">
         <is>
           <t>Verdict</t>
         </is>
       </c>
-      <c r="C1" s="52" t="inlineStr">
+      <c r="C1" s="57" t="inlineStr">
         <is>
           <t>Trades</t>
         </is>
       </c>
-      <c r="D1" s="52" t="inlineStr">
+      <c r="D1" s="57" t="inlineStr">
         <is>
           <t>Win %</t>
         </is>
       </c>
-      <c r="E1" s="52" t="inlineStr">
+      <c r="E1" s="57" t="inlineStr">
         <is>
           <t>Net P&amp;L</t>
         </is>
       </c>
-      <c r="F1" s="52" t="inlineStr">
+      <c r="F1" s="57" t="inlineStr">
         <is>
           <t>Avg/trade</t>
         </is>
       </c>
-      <c r="G1" s="52" t="inlineStr">
+      <c r="G1" s="57" t="inlineStr">
         <is>
           <t>Best</t>
         </is>
       </c>
-      <c r="H1" s="52" t="inlineStr">
+      <c r="H1" s="57" t="inlineStr">
         <is>
           <t>Worst</t>
         </is>
       </c>
-      <c r="I1" s="52" t="inlineStr">
+      <c r="I1" s="57" t="inlineStr">
         <is>
           <t>Avg peak %</t>
         </is>
       </c>
-      <c r="J1" s="52" t="inlineStr">
+      <c r="J1" s="57" t="inlineStr">
         <is>
           <t>Avg trough %</t>
         </is>
       </c>
-      <c r="K1" s="52" t="inlineStr">
+      <c r="K1" s="57" t="inlineStr">
         <is>
           <t>Days</t>
         </is>
       </c>
-      <c r="L1" s="52" t="inlineStr">
+      <c r="L1" s="57" t="inlineStr">
         <is>
           <t>Pre-8/19 trades*</t>
         </is>
       </c>
-      <c r="M1" s="52" t="inlineStr">
+      <c r="M1" s="57" t="inlineStr">
         <is>
           <t>Rooms</t>
         </is>
@@ -798,26 +806,26 @@
       <c r="C2" s="24" t="n">
         <v>9</v>
       </c>
-      <c r="D2" s="28" t="n">
+      <c r="D2" s="58" t="n">
         <v>0.3333</v>
       </c>
-      <c r="E2" s="53" t="n">
+      <c r="E2" s="59" t="n">
         <v>678</v>
       </c>
-      <c r="F2" s="53" t="n">
+      <c r="F2" s="60" t="n">
         <v>75.33</v>
       </c>
-      <c r="G2" s="53" t="n">
+      <c r="G2" s="60" t="n">
         <v>590</v>
       </c>
-      <c r="H2" s="54" t="n">
+      <c r="H2" s="60" t="n">
         <v>-37</v>
       </c>
       <c r="I2" s="24" t="n">
         <v>-1.8145</v>
       </c>
       <c r="J2" s="24" t="n">
-        <v>-1.85975</v>
+        <v>-1.8598</v>
       </c>
       <c r="K2" s="24" t="n">
         <v>6</v>
@@ -845,19 +853,19 @@
       <c r="C3" s="24" t="n">
         <v>2</v>
       </c>
-      <c r="D3" s="28" t="n">
+      <c r="D3" s="58" t="n">
         <v>1</v>
       </c>
-      <c r="E3" s="53" t="n">
+      <c r="E3" s="59" t="n">
         <v>252</v>
       </c>
-      <c r="F3" s="53" t="n">
+      <c r="F3" s="60" t="n">
         <v>126</v>
       </c>
-      <c r="G3" s="53" t="n">
+      <c r="G3" s="60" t="n">
         <v>217</v>
       </c>
-      <c r="H3" s="53" t="n">
+      <c r="H3" s="60" t="n">
         <v>35</v>
       </c>
       <c r="I3" s="24" t="n">
@@ -892,19 +900,19 @@
       <c r="C4" s="24" t="n">
         <v>12</v>
       </c>
-      <c r="D4" s="28" t="n">
+      <c r="D4" s="58" t="n">
         <v>0.25</v>
       </c>
-      <c r="E4" s="53" t="n">
+      <c r="E4" s="59" t="n">
         <v>223</v>
       </c>
-      <c r="F4" s="53" t="n">
+      <c r="F4" s="60" t="n">
         <v>18.58</v>
       </c>
-      <c r="G4" s="53" t="n">
+      <c r="G4" s="60" t="n">
         <v>420</v>
       </c>
-      <c r="H4" s="54" t="n">
+      <c r="H4" s="60" t="n">
         <v>-112</v>
       </c>
       <c r="I4" s="24" t="n">
@@ -939,19 +947,19 @@
       <c r="C5" s="24" t="n">
         <v>3</v>
       </c>
-      <c r="D5" s="28" t="n">
+      <c r="D5" s="58" t="n">
         <v>0.3333</v>
       </c>
-      <c r="E5" s="53" t="n">
+      <c r="E5" s="59" t="n">
         <v>197</v>
       </c>
-      <c r="F5" s="53" t="n">
+      <c r="F5" s="60" t="n">
         <v>65.67</v>
       </c>
-      <c r="G5" s="53" t="n">
+      <c r="G5" s="60" t="n">
         <v>209</v>
       </c>
-      <c r="H5" s="54" t="n">
+      <c r="H5" s="60" t="n">
         <v>-12</v>
       </c>
       <c r="I5" s="24" t="n">
@@ -986,19 +994,19 @@
       <c r="C6" s="24" t="n">
         <v>3</v>
       </c>
-      <c r="D6" s="28" t="n">
+      <c r="D6" s="58" t="n">
         <v>0.3333</v>
       </c>
-      <c r="E6" s="53" t="n">
+      <c r="E6" s="59" t="n">
         <v>39</v>
       </c>
-      <c r="F6" s="53" t="n">
+      <c r="F6" s="60" t="n">
         <v>13</v>
       </c>
-      <c r="G6" s="53" t="n">
+      <c r="G6" s="60" t="n">
         <v>53</v>
       </c>
-      <c r="H6" s="54" t="n">
+      <c r="H6" s="60" t="n">
         <v>-11</v>
       </c>
       <c r="I6" s="24" t="n"/>
@@ -1029,19 +1037,19 @@
       <c r="C7" s="24" t="n">
         <v>1</v>
       </c>
-      <c r="D7" s="28" t="n">
+      <c r="D7" s="58" t="n">
         <v>1</v>
       </c>
-      <c r="E7" s="53" t="n">
+      <c r="E7" s="59" t="n">
         <v>27</v>
       </c>
-      <c r="F7" s="53" t="n">
+      <c r="F7" s="60" t="n">
         <v>27</v>
       </c>
-      <c r="G7" s="53" t="n">
+      <c r="G7" s="60" t="n">
         <v>27</v>
       </c>
-      <c r="H7" s="53" t="n">
+      <c r="H7" s="60" t="n">
         <v>27</v>
       </c>
       <c r="I7" s="24" t="n"/>
@@ -1072,19 +1080,19 @@
       <c r="C8" s="24" t="n">
         <v>1</v>
       </c>
-      <c r="D8" s="28" t="n">
+      <c r="D8" s="58" t="n">
         <v>1</v>
       </c>
-      <c r="E8" s="53" t="n">
+      <c r="E8" s="59" t="n">
         <v>24</v>
       </c>
-      <c r="F8" s="53" t="n">
+      <c r="F8" s="60" t="n">
         <v>24</v>
       </c>
-      <c r="G8" s="53" t="n">
+      <c r="G8" s="60" t="n">
         <v>24</v>
       </c>
-      <c r="H8" s="53" t="n">
+      <c r="H8" s="60" t="n">
         <v>24</v>
       </c>
       <c r="I8" s="24" t="n"/>
@@ -1115,19 +1123,19 @@
       <c r="C9" s="24" t="n">
         <v>2</v>
       </c>
-      <c r="D9" s="28" t="n">
+      <c r="D9" s="58" t="n">
         <v>0.5</v>
       </c>
-      <c r="E9" s="53" t="n">
+      <c r="E9" s="59" t="n">
         <v>20</v>
       </c>
-      <c r="F9" s="53" t="n">
+      <c r="F9" s="60" t="n">
         <v>10</v>
       </c>
-      <c r="G9" s="53" t="n">
+      <c r="G9" s="60" t="n">
         <v>49</v>
       </c>
-      <c r="H9" s="54" t="n">
+      <c r="H9" s="60" t="n">
         <v>-29</v>
       </c>
       <c r="I9" s="24" t="n">
@@ -1162,19 +1170,19 @@
       <c r="C10" s="24" t="n">
         <v>1</v>
       </c>
-      <c r="D10" s="28" t="n">
+      <c r="D10" s="58" t="n">
         <v>1</v>
       </c>
-      <c r="E10" s="53" t="n">
+      <c r="E10" s="59" t="n">
         <v>15</v>
       </c>
-      <c r="F10" s="53" t="n">
+      <c r="F10" s="60" t="n">
         <v>15</v>
       </c>
-      <c r="G10" s="53" t="n">
+      <c r="G10" s="60" t="n">
         <v>15</v>
       </c>
-      <c r="H10" s="53" t="n">
+      <c r="H10" s="60" t="n">
         <v>15</v>
       </c>
       <c r="I10" s="24" t="n"/>
@@ -1205,26 +1213,26 @@
       <c r="C11" s="24" t="n">
         <v>7</v>
       </c>
-      <c r="D11" s="28" t="n">
+      <c r="D11" s="58" t="n">
         <v>0.2857</v>
       </c>
-      <c r="E11" s="53" t="n">
+      <c r="E11" s="59" t="n">
         <v>5</v>
       </c>
-      <c r="F11" s="53" t="n">
+      <c r="F11" s="60" t="n">
         <v>0.71</v>
       </c>
-      <c r="G11" s="53" t="n">
+      <c r="G11" s="60" t="n">
         <v>12</v>
       </c>
-      <c r="H11" s="54" t="n">
+      <c r="H11" s="60" t="n">
         <v>-9</v>
       </c>
       <c r="I11" s="24" t="n">
-        <v>0.07700000000000001</v>
+        <v>0.077</v>
       </c>
       <c r="J11" s="24" t="n">
-        <v>-0.05574999999999999</v>
+        <v>-0.0557</v>
       </c>
       <c r="K11" s="24" t="n">
         <v>4</v>
@@ -1252,19 +1260,19 @@
       <c r="C12" s="24" t="n">
         <v>2</v>
       </c>
-      <c r="D12" s="28" t="n">
+      <c r="D12" s="58" t="n">
         <v>0.5</v>
       </c>
-      <c r="E12" s="53" t="n">
+      <c r="E12" s="59" t="n">
         <v>2</v>
       </c>
-      <c r="F12" s="53" t="n">
+      <c r="F12" s="60" t="n">
         <v>1</v>
       </c>
-      <c r="G12" s="53" t="n">
+      <c r="G12" s="60" t="n">
         <v>27</v>
       </c>
-      <c r="H12" s="54" t="n">
+      <c r="H12" s="60" t="n">
         <v>-25</v>
       </c>
       <c r="I12" s="24" t="n">
@@ -1293,25 +1301,25 @@
       </c>
       <c r="B13" s="24" t="inlineStr">
         <is>
-          <t>WATCH</t>
+          <t>AVOID</t>
         </is>
       </c>
       <c r="C13" s="24" t="n">
         <v>4</v>
       </c>
-      <c r="D13" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="E13" s="55" t="n">
-        <v>0</v>
-      </c>
-      <c r="F13" s="55" t="n">
-        <v>0</v>
-      </c>
-      <c r="G13" s="55" t="n">
-        <v>0</v>
-      </c>
-      <c r="H13" s="55" t="n">
+      <c r="D13" s="58" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" s="61" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="60" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" s="60" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="60" t="n">
         <v>0</v>
       </c>
       <c r="I13" s="24" t="n"/>
@@ -1336,25 +1344,25 @@
       </c>
       <c r="B14" s="24" t="inlineStr">
         <is>
-          <t>WATCH</t>
+          <t>AVOID</t>
         </is>
       </c>
       <c r="C14" s="24" t="n">
         <v>5</v>
       </c>
-      <c r="D14" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="E14" s="55" t="n">
-        <v>0</v>
-      </c>
-      <c r="F14" s="55" t="n">
-        <v>0</v>
-      </c>
-      <c r="G14" s="55" t="n">
-        <v>0</v>
-      </c>
-      <c r="H14" s="55" t="n">
+      <c r="D14" s="58" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" s="61" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="60" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="60" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" s="60" t="n">
         <v>0</v>
       </c>
       <c r="I14" s="24" t="n"/>
@@ -1385,19 +1393,19 @@
       <c r="C15" s="24" t="n">
         <v>1</v>
       </c>
-      <c r="D15" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="E15" s="54" t="n">
+      <c r="D15" s="58" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" s="61" t="n">
         <v>-4</v>
       </c>
-      <c r="F15" s="54" t="n">
+      <c r="F15" s="60" t="n">
         <v>-4</v>
       </c>
-      <c r="G15" s="54" t="n">
+      <c r="G15" s="60" t="n">
         <v>-4</v>
       </c>
-      <c r="H15" s="54" t="n">
+      <c r="H15" s="60" t="n">
         <v>-4</v>
       </c>
       <c r="I15" s="24" t="n">
@@ -1432,19 +1440,19 @@
       <c r="C16" s="24" t="n">
         <v>1</v>
       </c>
-      <c r="D16" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="E16" s="54" t="n">
+      <c r="D16" s="58" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" s="61" t="n">
         <v>-10</v>
       </c>
-      <c r="F16" s="54" t="n">
+      <c r="F16" s="60" t="n">
         <v>-10</v>
       </c>
-      <c r="G16" s="54" t="n">
+      <c r="G16" s="60" t="n">
         <v>-10</v>
       </c>
-      <c r="H16" s="54" t="n">
+      <c r="H16" s="60" t="n">
         <v>-10</v>
       </c>
       <c r="I16" s="24" t="n"/>
@@ -1464,101 +1472,97 @@
     <row r="17">
       <c r="A17" s="24" t="inlineStr">
         <is>
-          <t>ZTRADEZ BOT</t>
+          <t>Bullwinkle</t>
         </is>
       </c>
       <c r="B17" s="24" t="inlineStr">
         <is>
-          <t>WATCH (small sample)</t>
+          <t>AVOID</t>
         </is>
       </c>
       <c r="C17" s="24" t="n">
-        <v>2</v>
-      </c>
-      <c r="D17" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="E17" s="54" t="n">
-        <v>-12.17</v>
-      </c>
-      <c r="F17" s="54" t="n">
-        <v>-6.09</v>
-      </c>
-      <c r="G17" s="54" t="n">
-        <v>-2.12</v>
-      </c>
-      <c r="H17" s="54" t="n">
-        <v>-10.05</v>
+        <v>9</v>
+      </c>
+      <c r="D17" s="58" t="n">
+        <v>0.3333</v>
+      </c>
+      <c r="E17" s="61" t="n">
+        <v>-16</v>
+      </c>
+      <c r="F17" s="60" t="n">
+        <v>-1.78</v>
+      </c>
+      <c r="G17" s="60" t="n">
+        <v>120</v>
+      </c>
+      <c r="H17" s="60" t="n">
+        <v>-45</v>
       </c>
       <c r="I17" s="24" t="n">
-        <v>-7.95</v>
+        <v>4.027</v>
       </c>
       <c r="J17" s="24" t="n">
-        <v>-10.9</v>
+        <v>-0.068</v>
       </c>
       <c r="K17" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="L17" s="24" t="n">
         <v>1</v>
       </c>
-      <c r="L17" s="24" t="n">
-        <v>0</v>
-      </c>
       <c r="M17" s="24" t="inlineStr">
         <is>
-          <t>ZT (1334236429655740457)</t>
+          <t>ZT scalps / ZT top-flow</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="24" t="inlineStr">
         <is>
-          <t>Bullwinkle</t>
+          <t>Shakira T</t>
         </is>
       </c>
       <c r="B18" s="24" t="inlineStr">
         <is>
-          <t>BENCH</t>
+          <t>WATCH (small sample)</t>
         </is>
       </c>
       <c r="C18" s="24" t="n">
-        <v>9</v>
-      </c>
-      <c r="D18" s="28" t="n">
-        <v>0.3333</v>
-      </c>
-      <c r="E18" s="54" t="n">
-        <v>-16</v>
-      </c>
-      <c r="F18" s="54" t="n">
-        <v>-1.78</v>
-      </c>
-      <c r="G18" s="53" t="n">
-        <v>120</v>
-      </c>
-      <c r="H18" s="54" t="n">
-        <v>-45</v>
-      </c>
-      <c r="I18" s="24" t="n">
-        <v>4.027</v>
-      </c>
-      <c r="J18" s="24" t="n">
-        <v>-0.068</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="D18" s="58" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" s="61" t="n">
+        <v>-21</v>
+      </c>
+      <c r="F18" s="60" t="n">
+        <v>-21</v>
+      </c>
+      <c r="G18" s="60" t="n">
+        <v>-21</v>
+      </c>
+      <c r="H18" s="60" t="n">
+        <v>-21</v>
+      </c>
+      <c r="I18" s="24" t="n"/>
+      <c r="J18" s="24" t="n"/>
       <c r="K18" s="24" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="L18" s="24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M18" s="24" t="inlineStr">
         <is>
-          <t>ZT scalps; ZT top-flow</t>
+          <t>Option Alerts</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="24" t="inlineStr">
         <is>
-          <t>Shakira T</t>
+          <t>TradingTheTrend</t>
         </is>
       </c>
       <c r="B19" s="24" t="inlineStr">
@@ -1567,27 +1571,31 @@
         </is>
       </c>
       <c r="C19" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="D19" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="E19" s="54" t="n">
-        <v>-21</v>
-      </c>
-      <c r="F19" s="54" t="n">
-        <v>-21</v>
-      </c>
-      <c r="G19" s="54" t="n">
-        <v>-21</v>
-      </c>
-      <c r="H19" s="54" t="n">
-        <v>-21</v>
-      </c>
-      <c r="I19" s="24" t="n"/>
-      <c r="J19" s="24" t="n"/>
+        <v>2</v>
+      </c>
+      <c r="D19" s="58" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" s="61" t="n">
+        <v>-22</v>
+      </c>
+      <c r="F19" s="60" t="n">
+        <v>-11</v>
+      </c>
+      <c r="G19" s="60" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" s="60" t="n">
+        <v>-22</v>
+      </c>
+      <c r="I19" s="24" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="J19" s="24" t="n">
+        <v>-0.059</v>
+      </c>
       <c r="K19" s="24" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L19" s="24" t="n">
         <v>0</v>
@@ -1601,184 +1609,184 @@
     <row r="20">
       <c r="A20" s="24" t="inlineStr">
         <is>
-          <t>TradingTheTrend</t>
+          <t>are alerts</t>
         </is>
       </c>
       <c r="B20" s="24" t="inlineStr">
         <is>
-          <t>WATCH (small sample)</t>
+          <t>AVOID</t>
         </is>
       </c>
       <c r="C20" s="24" t="n">
-        <v>2</v>
-      </c>
-      <c r="D20" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="E20" s="54" t="n">
-        <v>-22</v>
-      </c>
-      <c r="F20" s="54" t="n">
-        <v>-11</v>
-      </c>
-      <c r="G20" s="55" t="n">
-        <v>0</v>
-      </c>
-      <c r="H20" s="54" t="n">
-        <v>-22</v>
+        <v>3</v>
+      </c>
+      <c r="D20" s="58" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" s="61" t="n">
+        <v>-47</v>
+      </c>
+      <c r="F20" s="60" t="n">
+        <v>-15.67</v>
+      </c>
+      <c r="G20" s="60" t="n">
+        <v>0</v>
+      </c>
+      <c r="H20" s="60" t="n">
+        <v>-42</v>
       </c>
       <c r="I20" s="24" t="n">
-        <v>0.02</v>
+        <v>1.8573</v>
       </c>
       <c r="J20" s="24" t="n">
-        <v>-0.059</v>
+        <v>-1.3577</v>
       </c>
       <c r="K20" s="24" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L20" s="24" t="n">
         <v>0</v>
       </c>
       <c r="M20" s="24" t="inlineStr">
         <is>
-          <t>Option Alerts</t>
+          <t>ZT opt-2</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="24" t="inlineStr">
         <is>
-          <t>are alerts</t>
+          <t>MR.TOPHAT</t>
         </is>
       </c>
       <c r="B21" s="24" t="inlineStr">
         <is>
-          <t>BENCH</t>
+          <t>AVOID</t>
         </is>
       </c>
       <c r="C21" s="24" t="n">
-        <v>3</v>
-      </c>
-      <c r="D21" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="E21" s="54" t="n">
-        <v>-47</v>
-      </c>
-      <c r="F21" s="54" t="n">
-        <v>-15.67</v>
-      </c>
-      <c r="G21" s="55" t="n">
-        <v>0</v>
-      </c>
-      <c r="H21" s="54" t="n">
-        <v>-42</v>
+        <v>4</v>
+      </c>
+      <c r="D21" s="58" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E21" s="61" t="n">
+        <v>-48</v>
+      </c>
+      <c r="F21" s="60" t="n">
+        <v>-12</v>
+      </c>
+      <c r="G21" s="60" t="n">
+        <v>33</v>
+      </c>
+      <c r="H21" s="60" t="n">
+        <v>-50</v>
       </c>
       <c r="I21" s="24" t="n">
-        <v>1.857333333333333</v>
+        <v>-0.032</v>
       </c>
       <c r="J21" s="24" t="n">
-        <v>-1.357666666666667</v>
+        <v>-0.0955</v>
       </c>
       <c r="K21" s="24" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L21" s="24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M21" s="24" t="inlineStr">
         <is>
-          <t>ZT opt-2</t>
+          <t>MR.TOPHAT</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="24" t="inlineStr">
         <is>
-          <t>MR.TOPHAT</t>
+          <t>👑KingBeeAri🐝</t>
         </is>
       </c>
       <c r="B22" s="24" t="inlineStr">
         <is>
-          <t>BENCH</t>
+          <t>WATCH (small sample)</t>
         </is>
       </c>
       <c r="C22" s="24" t="n">
-        <v>4</v>
-      </c>
-      <c r="D22" s="28" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="E22" s="54" t="n">
-        <v>-48</v>
-      </c>
-      <c r="F22" s="54" t="n">
-        <v>-12</v>
-      </c>
-      <c r="G22" s="53" t="n">
-        <v>33</v>
-      </c>
-      <c r="H22" s="54" t="n">
-        <v>-50</v>
-      </c>
-      <c r="I22" s="24" t="n">
-        <v>-0.032</v>
-      </c>
-      <c r="J22" s="24" t="n">
-        <v>-0.0955</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="D22" s="58" t="n">
+        <v>0</v>
+      </c>
+      <c r="E22" s="61" t="n">
+        <v>-75</v>
+      </c>
+      <c r="F22" s="60" t="n">
+        <v>-75</v>
+      </c>
+      <c r="G22" s="60" t="n">
+        <v>-75</v>
+      </c>
+      <c r="H22" s="60" t="n">
+        <v>-75</v>
+      </c>
+      <c r="I22" s="24" t="n"/>
+      <c r="J22" s="24" t="n"/>
       <c r="K22" s="24" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L22" s="24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M22" s="24" t="inlineStr">
         <is>
-          <t>MR.TOPHAT</t>
+          <t>Honeydrip aristotle</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="24" t="inlineStr">
         <is>
-          <t>👑KingBeeAri🐝</t>
+          <t>ZTRADEZ BOT</t>
         </is>
       </c>
       <c r="B23" s="24" t="inlineStr">
         <is>
-          <t>WATCH (small sample)</t>
+          <t>AVOID</t>
         </is>
       </c>
       <c r="C23" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="D23" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="E23" s="54" t="n">
-        <v>-75</v>
-      </c>
-      <c r="F23" s="54" t="n">
-        <v>-75</v>
-      </c>
-      <c r="G23" s="54" t="n">
-        <v>-75</v>
-      </c>
-      <c r="H23" s="54" t="n">
-        <v>-75</v>
-      </c>
-      <c r="I23" s="24" t="n"/>
-      <c r="J23" s="24" t="n"/>
+        <v>6</v>
+      </c>
+      <c r="D23" s="58" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" s="61" t="n">
+        <v>-82.17</v>
+      </c>
+      <c r="F23" s="60" t="n">
+        <v>-13.7</v>
+      </c>
+      <c r="G23" s="60" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" s="60" t="n">
+        <v>-50</v>
+      </c>
+      <c r="I23" s="24" t="n">
+        <v>-4.4</v>
+      </c>
+      <c r="J23" s="24" t="n">
+        <v>-20.62</v>
+      </c>
       <c r="K23" s="24" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L23" s="24" t="n">
         <v>0</v>
       </c>
       <c r="M23" s="24" t="inlineStr">
         <is>
-          <t>Honeydrip aristotle</t>
+          <t>ZT (1334236429655740457)</t>
         </is>
       </c>
     </row>
@@ -1790,29 +1798,29 @@
       </c>
       <c r="B24" s="24" t="inlineStr">
         <is>
-          <t>BENCH</t>
+          <t>AVOID</t>
         </is>
       </c>
       <c r="C24" s="24" t="n">
         <v>3</v>
       </c>
-      <c r="D24" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="E24" s="54" t="n">
+      <c r="D24" s="58" t="n">
+        <v>0</v>
+      </c>
+      <c r="E24" s="61" t="n">
         <v>-195</v>
       </c>
-      <c r="F24" s="54" t="n">
+      <c r="F24" s="60" t="n">
         <v>-65</v>
       </c>
-      <c r="G24" s="54" t="n">
+      <c r="G24" s="60" t="n">
         <v>-44</v>
       </c>
-      <c r="H24" s="54" t="n">
+      <c r="H24" s="60" t="n">
         <v>-96</v>
       </c>
       <c r="I24" s="24" t="n">
-        <v>0.009000000000000006</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="J24" s="24" t="n">
         <v>-0.225</v>
@@ -1830,107 +1838,135 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="56" t="inlineStr">
+      <c r="A26" s="23" t="inlineStr">
         <is>
           <t>* Trades before 8/19 predate the ledger fix — those P&amp;L numbers can run hot. 8/19 onward is broker-verified (FIFO on real fills).</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="56" t="inlineStr">
+      <c r="A27" s="23" t="inlineStr">
         <is>
           <t>* 8/24: days/2026-08-24.json missed 5 bot trades entirely — those rows are rebuilt from broker fills, not the ledger.</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="56" t="inlineStr">
+      <c r="A28" s="23" t="inlineStr">
         <is>
           <t>* 8/25: same ledger-miss bug — UBER x3 (-$75) never reached days/2026-08-25.json or journal.csv. Rebuilt from broker fills.</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="56" t="inlineStr">
+      <c r="A29" s="23" t="inlineStr">
         <is>
           <t>* 8/25: a phantom NVDA +$70 row and a duplicate SPCX -$10 row were dropped — neither had a broker fill behind it.</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="56" t="inlineStr">
+      <c r="A30" s="23" t="inlineStr">
         <is>
           <t>* 8/26: bridge was shut down ~10:37 AM ET — days/2026-08-26.json held ONE row (an open QQQ). All 5 caller trades rebuilt from broker fills.</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="56" t="inlineStr">
+      <c r="A31" s="23" t="inlineStr">
         <is>
           <t>* 8/26: PHANTOM — TSLA 350P bracket stop filled @4.70 (-$45) at 09:48:22, but the bot booked '+$70, you closed it yourself' at 09:53:18. $115 swing, corrected.</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="56" t="inlineStr">
+      <c r="A32" s="23" t="inlineStr">
         <is>
           <t>* 8/26: TSLA 345P (-$39, Bullwinkle) never reached the ledger at all — no FILLED and no exit line. Broker-only.</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="56" t="inlineStr">
+      <c r="A33" s="23" t="inlineStr">
         <is>
           <t>* 8/26: SLV and CDE closed on the bot's OWN resting GTC stops, but were logged 'you closed it yourself' at -$5/-$10. True -$42/-$25.</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="56" t="inlineStr">
+      <c r="A34" s="23" t="inlineStr">
         <is>
           <t>* 8/27: bridge was OFF the entire session. Zero caller trades. Every 8/27 fill is Gian's own and is excluded from this scoreboard.</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="56" t="inlineStr">
+      <c r="A35" s="23" t="inlineStr">
         <is>
           <t>* 8/28: the bot placed ZERO orders. All 4 option opens were rejected by Webull HTTP 417 "your account is not eligible to trade options now" (SPCX, ABT, WFC, PBR). Those $0 lines are a broker permissions block, not caller skill.</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="56" t="inlineStr">
+      <c r="A36" s="23" t="inlineStr">
         <is>
           <t>* 8/28: MNQ (Market Guru) — Webull leg routed at a non-futures account, no fill in 90s; Topstep refused ("Auto OCO Brackets" not enabled); NinjaTrader filled it with NO stop (no ATM template set).</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="56" t="inlineStr">
+      <c r="A37" s="23" t="inlineStr">
         <is>
           <t>* 8/28: execution.mode = dryrun and no room flipped REAL. Every 8/28 broker fill is Gian's own and is excluded from this scoreboard.</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="56" t="inlineStr">
+      <c r="A38" s="23" t="inlineStr">
         <is>
           <t>* 8/31: PHANTOM — bot adopted Gian's SPY 765C at 11:19:24; he sold it at the broker 43s later. Bot carried the ghost 3h22m, then ran a failed sell/stop loop (417 'insufficient underlying') and booked $0. Gian trade, not a caller trade — excluded from caller stats.</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="56" t="inlineStr">
+      <c r="A39" s="23" t="inlineStr">
         <is>
           <t>* 8/31: LEDGER SHORT — bot adopted only 2 of Gian's 4 SPY 766C and booked +$36; broker FIFO on all 4 = +$83.62. Gian trade, excluded from caller stats.</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="56" t="inlineStr">
+      <c r="A40" s="23" t="inlineStr">
         <is>
           <t>* 8/31: STOP-WARN — S 22.5C 9/18 swing carries overnight with the broker STOP_LOSS leg CANCELLED (DAY order, died at the close). Local watchdog only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="23" t="inlineStr">
+        <is>
+          <t>* 9/01: LEDGER MISS x4 - QQQ 706P (-$31), SPY 760P (+$17), QQQ 713C (-$24) and QQQ 708C x13 (+$156) never reached days/2026-09-01.json. All Gian's own, excluded from caller stats, rebuilt from broker fills.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="23" t="inlineStr">
+        <is>
+          <t>* 9/01: All THREE ZT mashup exits closed on the bot's OWN resting Webull stop and were booked $0 by the ledger (true -$50 / -$12 / -$8). Same 'sold at a price I never saw' path as 8/26 SLV &amp; CDE - the corrected numbers here are broker FIFO.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="23" t="inlineStr">
+        <is>
+          <t>* 9/01: STOP-WARN - FLR 57.5C 9/18 swing carries overnight with the broker STOP_LOSS leg CANCELLED (DAY order, died at the close). Second night running after S on 8/31. Local -25% watcher only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="23" t="inlineStr">
+        <is>
+          <t>* 9/01: caller names are now readable in the raw text of ZT mashup calls (The Market Bishop = S and FLR, Jpm Options = SPY 764P). Still booked under 'ZTRADEZ BOT' for continuity - worth splitting into real per-caller rows.</t>
         </is>
       </c>
     </row>
@@ -1945,7 +1981,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J80"/>
+  <dimension ref="A1:J84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4940,7 +4976,7 @@
         <v>22.5</v>
       </c>
       <c r="E80" s="25" t="n">
-        <v>-10.05</v>
+        <v>0</v>
       </c>
       <c r="F80" s="24" t="n">
         <v>-5.9</v>
@@ -4948,15 +4984,177 @@
       <c r="G80" s="24" t="n">
         <v>-11.8</v>
       </c>
-      <c r="H80" s="24" t="inlineStr">
-        <is>
-          <t>OPEN overnight swing — broker stop CANCELLED at close, mark to bid 0.75</t>
+      <c r="H80" s="56" t="inlineStr">
+        <is>
+          <t>superseded - closed 9/01 at -50.00 (see 9/01 row); 8/31 mark-to-bid zeroed to avoid double-count</t>
         </is>
       </c>
       <c r="I80" s="24" t="b">
         <v>1</v>
       </c>
       <c r="J80" s="24" t="inlineStr">
+        <is>
+          <t>ZT (1334236429655740457)</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B81" s="24" t="inlineStr">
+        <is>
+          <t>ZTRADEZ BOT</t>
+        </is>
+      </c>
+      <c r="C81" s="24" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="D81" s="24" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="E81" s="60" t="n">
+        <v>-50</v>
+      </c>
+      <c r="F81" s="24" t="n"/>
+      <c r="G81" s="24" t="n">
+        <v>-58.8</v>
+      </c>
+      <c r="H81" s="24" t="inlineStr">
+        <is>
+          <t>bot's own GTC stop-limit filled at broker 12:36:03 (logged as a hand close, booked $0)</t>
+        </is>
+      </c>
+      <c r="I81" s="24" t="b">
+        <v>1</v>
+      </c>
+      <c r="J81" s="24" t="inlineStr">
+        <is>
+          <t>ZT (1334236429655740457)</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B82" s="24" t="inlineStr">
+        <is>
+          <t>ZTRADEZ BOT</t>
+        </is>
+      </c>
+      <c r="C82" s="24" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="D82" s="24" t="n">
+        <v>764</v>
+      </c>
+      <c r="E82" s="60" t="n">
+        <v>-12</v>
+      </c>
+      <c r="F82" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="G82" s="24" t="n">
+        <v>-11.5</v>
+      </c>
+      <c r="H82" s="24" t="inlineStr">
+        <is>
+          <t>bot resting stop-limit filled 10:47:45 (booked $0)</t>
+        </is>
+      </c>
+      <c r="I82" s="24" t="b">
+        <v>0</v>
+      </c>
+      <c r="J82" s="24" t="inlineStr">
+        <is>
+          <t>ZT (1334236429655740457)</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B83" s="24" t="inlineStr">
+        <is>
+          <t>ZTRADEZ BOT</t>
+        </is>
+      </c>
+      <c r="C83" s="24" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="D83" s="24" t="n">
+        <v>764</v>
+      </c>
+      <c r="E83" s="60" t="n">
+        <v>-8</v>
+      </c>
+      <c r="F83" s="24" t="n">
+        <v>-2.7</v>
+      </c>
+      <c r="G83" s="24" t="n">
+        <v>-11</v>
+      </c>
+      <c r="H83" s="24" t="inlineStr">
+        <is>
+          <t>bot resting stop-limit filled 12:14:15 (booked $0)</t>
+        </is>
+      </c>
+      <c r="I83" s="24" t="b">
+        <v>0</v>
+      </c>
+      <c r="J83" s="24" t="inlineStr">
+        <is>
+          <t>ZT (1334236429655740457)</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="24" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B84" s="24" t="inlineStr">
+        <is>
+          <t>ZTRADEZ BOT</t>
+        </is>
+      </c>
+      <c r="C84" s="24" t="inlineStr">
+        <is>
+          <t>FLR</t>
+        </is>
+      </c>
+      <c r="D84" s="24" t="n">
+        <v>57.5</v>
+      </c>
+      <c r="E84" s="60" t="n">
+        <v>0</v>
+      </c>
+      <c r="F84" s="24" t="n"/>
+      <c r="G84" s="24" t="n"/>
+      <c r="H84" s="24" t="inlineStr">
+        <is>
+          <t>OPEN overnight swing - broker stop CANCELLED at close; mark to bid 1.725 = +8.50 unrealised</t>
+        </is>
+      </c>
+      <c r="I84" s="24" t="b">
+        <v>1</v>
+      </c>
+      <c r="J84" s="24" t="inlineStr">
         <is>
           <t>ZT (1334236429655740457)</t>
         </is>

</xml_diff>